<commit_message>
visor 2 pestanas + columna TIPO
</commit_message>
<xml_diff>
--- a/RESPUESTAS CORRECTAS PROYECTO JULIANA.xlsx
+++ b/RESPUESTAS CORRECTAS PROYECTO JULIANA.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16212F19-C719-475C-A0C4-6F5566BB112E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{732323EC-F4F5-435F-AF0C-C0574B451834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{53EC3F7E-E675-4FE9-9D45-980DAA55F6C0}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{53EC3F7E-E675-4FE9-9D45-980DAA55F6C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$D$191</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">

</xml_diff>

<commit_message>
actualiza acumulados 19/06/2026 12:11
</commit_message>
<xml_diff>
--- a/RESPUESTAS CORRECTAS PROYECTO JULIANA.xlsx
+++ b/RESPUESTAS CORRECTAS PROYECTO JULIANA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BFF660B-F9A5-407E-82F7-6A416BAC2870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE94278E-6675-4D36-A5FA-D6D4A8EA5504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{53EC3F7E-E675-4FE9-9D45-980DAA55F6C0}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="11">
   <si>
     <t>D</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t>REGUNTA NÚMERO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B o C </t>
   </si>
 </sst>
 </file>
@@ -1596,7 +1599,7 @@
         <v>2</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
@@ -2268,7 +2271,7 @@
         <v>10</v>
       </c>
       <c r="D121" s="5" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>